<commit_message>
refactor: implement unified digital twin runner with adaptive diagnostic bands and high-dimensional residual feature pipeline
</commit_message>
<xml_diff>
--- a/data/raw/engine_dataset/Data_vaibhav_colored.xlsx
+++ b/data/raw/engine_dataset/Data_vaibhav_colored.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwprod-my.sharepoint.com/personal/sgupta278_wisc_edu/Documents/Laptop data/A Saurabh/Startup/VIrtual Sensor/Data/Fw_ Follow-up_ Virtual Sensor Dataset and Recommended Readings/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sherry\Desktop\digital-twin-engine-virtual-sensor-research\data\raw\engine_dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="11_6435D1037EC715DFD19D6980FA5775EEB0320D8A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{491C2350-FEAC-46CE-AEB9-D54B876A9890}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B75EFE7A-8DC9-417E-934D-6A934619CA51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2490" yWindow="2295" windowWidth="23865" windowHeight="12480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="636" yWindow="3336" windowWidth="19008" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Virtual sensor" sheetId="2" r:id="rId1"/>
@@ -210,12 +210,19 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -264,7 +271,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -565,10 +572,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{247FD156-8DCD-4301-8DC7-B7BAD595FC4D}">
   <dimension ref="A1:AR219"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="28" max="28" width="14.140625" customWidth="1"/>
-    <col min="29" max="29" width="10.5703125" customWidth="1"/>
+    <col min="1" max="1" width="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="27" width="9" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="14.109375" customWidth="1"/>
+    <col min="29" max="29" width="10.5546875" customWidth="1"/>
+    <col min="30" max="33" width="9" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="35" max="38" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.25">
@@ -29918,6 +29931,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -29925,10 +29939,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AU219"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="31" max="31" width="14.140625" customWidth="1"/>
-    <col min="32" max="32" width="10.5703125" customWidth="1"/>
+    <col min="31" max="31" width="14.109375" customWidth="1"/>
+    <col min="32" max="32" width="10.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:47" x14ac:dyDescent="0.25">
@@ -61249,6 +61263,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>